<commit_message>
update meetingnote,WBS,feedbacknote(new),filelist add fold PRD displaydescript
</commit_message>
<xml_diff>
--- a/Final_Project_파일_관리_대장.xlsx
+++ b/Final_Project_파일_관리_대장.xlsx
@@ -6,7 +6,7 @@
     <sheet state="visible" name="파일관리" sheetId="1" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'파일관리'!$B$2:$Q$60</definedName>
+    <definedName hidden="1" localSheetId="0" name="_xlnm._FilterDatabase">'파일관리'!$B$2:$P$60</definedName>
   </definedNames>
   <calcPr/>
 </workbook>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="128">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="134">
   <si>
     <t>No.</t>
   </si>
@@ -72,9 +72,6 @@
     <t>생성일자</t>
   </si>
   <si>
-    <t>초안마감일자</t>
-  </si>
-  <si>
     <t>마감일자</t>
   </si>
   <si>
@@ -174,19 +171,19 @@
     <t>05</t>
   </si>
   <si>
-    <t>Final_Project_서비스 플로우차트v01</t>
+    <t>Final_Project_서비스 플로우차트</t>
   </si>
   <si>
     <t>AI 면접 프로그램에 대한 플로우 차트. 전체적인 흐름을
 도식화해서 표현함.</t>
   </si>
   <si>
+    <t>md</t>
+  </si>
+  <si>
     <t>검토중</t>
   </si>
   <si>
-    <t>AI 면접 통합 서비스 플로우차트v01.docx</t>
-  </si>
-  <si>
     <t>06</t>
   </si>
   <si>
@@ -217,9 +214,6 @@
     <t>프로젝트의 전체 범위를 최소 단위의 작업으로 쪼개어 '누가, 언제까지, 무엇을 개발할지'를 한눈에 볼 수 있도록 정리한 일정 및 자원 관리 문서</t>
   </si>
   <si>
-    <t>진희,혜현</t>
-  </si>
-  <si>
     <t>09</t>
   </si>
   <si>
@@ -298,16 +292,40 @@
     <t>17</t>
   </si>
   <si>
+    <t>Final_Project_기술 아키텍처</t>
+  </si>
+  <si>
     <t>18</t>
   </si>
   <si>
+    <t>Final_Project_QA</t>
+  </si>
+  <si>
+    <t>전체</t>
+  </si>
+  <si>
     <t>19</t>
   </si>
   <si>
+    <t>Final_Project_AI 아키텍처</t>
+  </si>
+  <si>
     <t>20</t>
   </si>
   <si>
+    <t>보고</t>
+  </si>
+  <si>
+    <t>피드백노트</t>
+  </si>
+  <si>
+    <t>각 문서를 읽고, 그에대한 피드백을 남기는 공유시트</t>
+  </si>
+  <si>
     <t>21</t>
+  </si>
+  <si>
+    <t>Final_Project_</t>
   </si>
   <si>
     <t>22</t>
@@ -428,7 +446,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="9">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -457,6 +475,22 @@
       <scheme val="minor"/>
     </font>
     <font/>
+    <font>
+      <b/>
+      <sz val="11.0"/>
+      <color rgb="FFFF0000"/>
+      <name val="Noto Sans KR"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color rgb="FFF79646"/>
+      <name val="Noto Sans KR"/>
+    </font>
+    <font>
+      <sz val="11.0"/>
+      <color theme="9"/>
+      <name val="Noto Sans KR"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -544,7 +578,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="22">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -581,11 +615,20 @@
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="5" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="6" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="7" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="8" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="9" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
+    <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="8" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
+    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -653,7 +696,36 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer">
+  <xdr:oneCellAnchor>
+    <xdr:from>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>3171825</xdr:colOff>
+      <xdr:row>59</xdr:row>
+      <xdr:rowOff>95250</xdr:rowOff>
+    </xdr:from>
+    <xdr:ext cx="6210300" cy="3514725"/>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="0" name="image1.png" title="이미지"/>
+        <xdr:cNvPicPr preferRelativeResize="0"/>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData fLocksWithSheet="0"/>
+  </xdr:oneCellAnchor>
+</xdr:wsDr>
 </file>
 
 <file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
@@ -872,10 +944,10 @@
     <col customWidth="1" min="10" max="10" width="10.71"/>
     <col customWidth="1" min="11" max="11" width="9.0"/>
     <col customWidth="1" min="12" max="12" width="10.0"/>
-    <col customWidth="1" min="13" max="15" width="12.0"/>
-    <col customWidth="1" min="16" max="16" width="44.0"/>
-    <col customWidth="1" min="17" max="17" width="36.0"/>
-    <col customWidth="1" min="18" max="27" width="8.71"/>
+    <col customWidth="1" min="13" max="14" width="12.0"/>
+    <col customWidth="1" min="15" max="15" width="44.0"/>
+    <col customWidth="1" min="16" max="16" width="36.0"/>
+    <col customWidth="1" min="17" max="26" width="8.71"/>
   </cols>
   <sheetData>
     <row r="1" ht="16.5" customHeight="1"/>
@@ -916,7 +988,7 @@
       <c r="M2" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="N2" s="2" t="s">
+      <c r="N2" s="1" t="s">
         <v>12</v>
       </c>
       <c r="O2" s="1" t="s">
@@ -925,266 +997,264 @@
       <c r="P2" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="Q2" s="1" t="s">
-        <v>15</v>
-      </c>
     </row>
     <row r="3" ht="28.5" customHeight="1">
       <c r="B3" s="3" t="s">
+        <v>15</v>
+      </c>
+      <c r="C3" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>17</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="E3" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="F3" s="3" t="s">
         <v>19</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G3" s="7" t="s">
+      <c r="H3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H3" s="7" t="s">
+      <c r="I3" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J3" s="3" t="s">
+      <c r="K3" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="K3" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L3" s="8"/>
       <c r="M3" s="9">
         <v>46317.0</v>
       </c>
       <c r="N3" s="9"/>
-      <c r="O3" s="9"/>
-      <c r="P3" s="6" t="str">
-        <f t="shared" ref="P3:P7" si="1">IF(D3="","",D3&amp;"_"&amp;IF(L3="",K3,L3)&amp;"."&amp;I3)</f>
+      <c r="O3" s="6" t="str">
+        <f t="shared" ref="O3:O60" si="1">IF(D3="","",D3&amp;"_"&amp;IF(L3="",K3,L3)&amp;"."&amp;I3)</f>
         <v>Final_Project_파일_관리_대장_0.01v.xlsx</v>
       </c>
-      <c r="Q3" s="6"/>
+      <c r="P3" s="6"/>
     </row>
     <row r="4" ht="28.5" customHeight="1">
       <c r="B4" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D4" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C4" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D4" s="5" t="s">
+      <c r="E4" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="E4" s="6" t="s">
+      <c r="F4" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G4" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H4" s="7" t="s">
         <v>28</v>
       </c>
-      <c r="F4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="G4" s="7" t="s">
+      <c r="I4" s="3" t="s">
         <v>22</v>
       </c>
-      <c r="H4" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I4" s="3" t="s">
+      <c r="J4" s="3" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="3" t="s">
+      <c r="K4" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="K4" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L4" s="8"/>
       <c r="M4" s="10">
         <v>46288.0</v>
       </c>
       <c r="N4" s="9"/>
-      <c r="O4" s="9"/>
-      <c r="P4" s="6" t="str">
+      <c r="O4" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_회의록_0.01v.xlsx</v>
       </c>
-      <c r="Q4" s="6"/>
-      <c r="S4" s="11"/>
+      <c r="P4" s="6"/>
+      <c r="R4" s="11"/>
+      <c r="S4" s="12"/>
       <c r="T4" s="12"/>
       <c r="U4" s="12"/>
       <c r="V4" s="12"/>
       <c r="W4" s="12"/>
-      <c r="X4" s="12"/>
-      <c r="Y4" s="13"/>
+      <c r="X4" s="13"/>
     </row>
     <row r="5" ht="28.5" customHeight="1">
       <c r="B5" s="3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C5" s="4" t="s">
         <v>30</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>31</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="E5" s="5" t="s">
         <v>32</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="F5" s="3" t="s">
+        <v>19</v>
+      </c>
+      <c r="G5" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="F5" s="3" t="s">
+      <c r="H5" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G5" s="7" t="s">
+      <c r="I5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="H5" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I5" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="J5" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K5" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="L5" s="8"/>
-      <c r="M5" s="9"/>
-      <c r="N5" s="10">
+      <c r="M5" s="10">
+        <v>46322.0</v>
+      </c>
+      <c r="N5" s="14">
         <v>46323.0</v>
       </c>
-      <c r="O5" s="9"/>
-      <c r="P5" s="6" t="str">
+      <c r="O5" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_PRD정의서_0.01v.docx</v>
       </c>
-      <c r="Q5" s="6"/>
-      <c r="S5" s="14"/>
-      <c r="Y5" s="15"/>
+      <c r="P5" s="6"/>
+      <c r="R5" s="15"/>
+      <c r="X5" s="16"/>
     </row>
     <row r="6" ht="28.5" customHeight="1">
       <c r="B6" s="3" t="s">
+        <v>35</v>
+      </c>
+      <c r="C6" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="C6" s="4" t="s">
+      <c r="D6" s="5" t="s">
         <v>37</v>
       </c>
-      <c r="D6" s="5" t="s">
+      <c r="E6" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>39</v>
-      </c>
       <c r="F6" s="3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G6" s="7" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="H6" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>35</v>
-      </c>
       <c r="J6" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="K6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="K6" s="7" t="s">
-        <v>25</v>
-      </c>
       <c r="L6" s="8"/>
-      <c r="M6" s="9"/>
-      <c r="N6" s="10">
+      <c r="M6" s="10">
         <v>46323.0</v>
       </c>
-      <c r="O6" s="9"/>
-      <c r="P6" s="6" t="str">
+      <c r="N6" s="17">
+        <v>46325.0</v>
+      </c>
+      <c r="O6" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_TRD정의서_0.01v.docx</v>
       </c>
-      <c r="Q6" s="6"/>
-      <c r="S6" s="14"/>
-      <c r="Y6" s="15"/>
+      <c r="P6" s="6"/>
+      <c r="R6" s="15"/>
+      <c r="X6" s="16"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="s">
+        <v>39</v>
+      </c>
+      <c r="C7" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D7" s="5" t="s">
         <v>40</v>
       </c>
-      <c r="C7" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" s="5" t="s">
+      <c r="E7" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="F7" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G7" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H7" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="F7" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G7" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7" s="7" t="s">
+      <c r="I7" s="4" t="s">
         <v>43</v>
-      </c>
-      <c r="I7" s="4" t="s">
-        <v>44</v>
       </c>
       <c r="J7" s="3"/>
       <c r="K7" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L7" s="8"/>
-      <c r="M7" s="9"/>
-      <c r="N7" s="10">
-        <v>46323.0</v>
-      </c>
-      <c r="O7" s="9"/>
-      <c r="P7" s="6" t="str">
+      <c r="M7" s="10">
+        <v>46322.0</v>
+      </c>
+      <c r="N7" s="17">
+        <v>46325.0</v>
+      </c>
+      <c r="O7" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_화면정의서_0.01v.pptx</v>
       </c>
-      <c r="Q7" s="6"/>
-      <c r="S7" s="14"/>
-      <c r="Y7" s="15"/>
+      <c r="P7" s="6"/>
+      <c r="R7" s="15"/>
+      <c r="X7" s="16"/>
     </row>
     <row r="8" ht="28.5" customHeight="1">
       <c r="B8" s="3" t="s">
+        <v>44</v>
+      </c>
+      <c r="C8" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="5" t="s">
         <v>45</v>
       </c>
-      <c r="C8" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D8" s="5" t="s">
+      <c r="E8" s="5" t="s">
         <v>46</v>
       </c>
-      <c r="E8" s="5" t="s">
+      <c r="F8" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G8" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H8" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I8" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="F8" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G8" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H8" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I8" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="J8" s="4" t="s">
         <v>48</v>
       </c>
       <c r="K8" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L8" s="8"/>
       <c r="M8" s="10">
@@ -1193,527 +1263,597 @@
       <c r="N8" s="10">
         <v>46322.0</v>
       </c>
-      <c r="O8" s="10">
-        <v>46322.0</v>
-      </c>
-      <c r="P8" s="5" t="s">
-        <v>49</v>
-      </c>
-      <c r="Q8" s="6"/>
-      <c r="S8" s="14"/>
-      <c r="Y8" s="15"/>
+      <c r="O8" s="5" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project_서비스 플로우차트_0.01v.md</v>
+      </c>
+      <c r="P8" s="6"/>
+      <c r="R8" s="15"/>
+      <c r="X8" s="16"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="s">
+        <v>49</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D9" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="C9" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D9" s="5" t="s">
+      <c r="E9" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="F9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G9" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H9" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I9" s="4" t="s">
         <v>52</v>
-      </c>
-      <c r="F9" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G9" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="H9" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="I9" s="4" t="s">
-        <v>53</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L9" s="8"/>
-      <c r="M9" s="9"/>
-      <c r="N9" s="9"/>
-      <c r="O9" s="9"/>
-      <c r="P9" s="6" t="str">
-        <f t="shared" ref="P9:P60" si="2">IF(D9="","",D9&amp;"_"&amp;IF(L9="",K9,L9)&amp;"."&amp;I9)</f>
+      <c r="M9" s="10">
+        <v>46325.0</v>
+      </c>
+      <c r="N9" s="17">
+        <v>46332.0</v>
+      </c>
+      <c r="O9" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_API 명세서_0.01v.yaml</v>
       </c>
-      <c r="Q9" s="6"/>
-      <c r="S9" s="14"/>
-      <c r="Y9" s="15"/>
+      <c r="P9" s="6"/>
+      <c r="R9" s="15"/>
+      <c r="X9" s="16"/>
     </row>
     <row r="10" ht="28.5" customHeight="1">
       <c r="B10" s="3" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="5" t="s">
         <v>54</v>
       </c>
-      <c r="C10" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D10" s="5" t="s">
+      <c r="E10" s="5" t="s">
         <v>55</v>
       </c>
-      <c r="E10" s="5" t="s">
-        <v>56</v>
-      </c>
       <c r="F10" s="4" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>21</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J10" s="3"/>
       <c r="K10" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L10" s="8"/>
-      <c r="M10" s="9"/>
-      <c r="N10" s="9"/>
-      <c r="O10" s="9"/>
-      <c r="P10" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M10" s="10">
+        <v>46323.0</v>
+      </c>
+      <c r="N10" s="17">
+        <v>46325.0</v>
+      </c>
+      <c r="O10" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_시나리오 기획서_0.01v.xlsx</v>
       </c>
-      <c r="Q10" s="6"/>
-      <c r="S10" s="14"/>
-      <c r="Y10" s="15"/>
+      <c r="P10" s="6"/>
+      <c r="R10" s="15"/>
+      <c r="X10" s="16"/>
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
+        <v>56</v>
+      </c>
+      <c r="C11" s="4" t="s">
+        <v>16</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C11" s="4" t="s">
-        <v>17</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>58</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>59</v>
-      </c>
       <c r="F11" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G11" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G11" s="7" t="s">
+      <c r="H11" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H11" s="7" t="s">
-        <v>60</v>
-      </c>
       <c r="I11" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="J11" s="4" t="s">
+      <c r="K11" s="7" t="s">
         <v>24</v>
-      </c>
-      <c r="K11" s="7" t="s">
-        <v>25</v>
       </c>
       <c r="L11" s="8"/>
       <c r="M11" s="10">
         <v>46322.0</v>
       </c>
-      <c r="N11" s="10">
-        <v>46322.0</v>
-      </c>
-      <c r="O11" s="9"/>
-      <c r="P11" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="N11" s="9"/>
+      <c r="O11" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_WBS_업무관리_0.01v.xlsx</v>
       </c>
-      <c r="Q11" s="6"/>
-      <c r="S11" s="14"/>
-      <c r="Y11" s="15"/>
+      <c r="P11" s="6"/>
+      <c r="R11" s="15"/>
+      <c r="X11" s="16"/>
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="B12" s="3" t="s">
+        <v>59</v>
+      </c>
+      <c r="C12" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>60</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>61</v>
       </c>
-      <c r="C12" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D12" s="5" t="s">
+      <c r="F12" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G12" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H12" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" s="4" t="s">
         <v>62</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="F12" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="G12" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H12" s="7" t="s">
-        <v>34</v>
-      </c>
-      <c r="I12" s="4" t="s">
-        <v>64</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L12" s="8"/>
-      <c r="M12" s="9"/>
-      <c r="N12" s="9"/>
-      <c r="O12" s="9"/>
-      <c r="P12" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M12" s="10">
+        <v>46325.0</v>
+      </c>
+      <c r="N12" s="17">
+        <v>46332.0</v>
+      </c>
+      <c r="O12" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_ERD_0.01v.png</v>
       </c>
-      <c r="Q12" s="6"/>
-      <c r="S12" s="14"/>
-      <c r="Y12" s="15"/>
+      <c r="P12" s="6"/>
+      <c r="R12" s="15"/>
+      <c r="X12" s="16"/>
     </row>
     <row r="13" ht="28.5" customHeight="1">
       <c r="B13" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="C13" s="4" t="s">
-        <v>37</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>66</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>67</v>
-      </c>
       <c r="F13" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G13" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H13" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G13" s="7" t="s">
+      <c r="I13" s="4" t="s">
         <v>22</v>
-      </c>
-      <c r="H13" s="7" t="s">
-        <v>21</v>
-      </c>
-      <c r="I13" s="4" t="s">
-        <v>23</v>
       </c>
       <c r="J13" s="3"/>
       <c r="K13" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L13" s="8"/>
-      <c r="M13" s="9"/>
-      <c r="N13" s="9"/>
-      <c r="O13" s="9"/>
-      <c r="P13" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M13" s="10">
+        <v>46325.0</v>
+      </c>
+      <c r="N13" s="17">
+        <v>46332.0</v>
+      </c>
+      <c r="O13" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_테이블 정의서_0.01v.xlsx</v>
       </c>
-      <c r="Q13" s="6"/>
-      <c r="S13" s="14"/>
-      <c r="Y13" s="15"/>
+      <c r="P13" s="6"/>
+      <c r="R13" s="15"/>
+      <c r="X13" s="16"/>
     </row>
     <row r="14" ht="28.5" customHeight="1">
       <c r="B14" s="3" t="s">
+        <v>66</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D14" s="5" t="s">
         <v>68</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="E14" s="5" t="s">
         <v>69</v>
       </c>
-      <c r="D14" s="5" t="s">
-        <v>70</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>71</v>
-      </c>
       <c r="F14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G14" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G14" s="7" t="s">
-        <v>21</v>
-      </c>
       <c r="H14" s="7" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="I14" s="4" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J14" s="3"/>
       <c r="K14" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L14" s="8"/>
-      <c r="M14" s="9"/>
-      <c r="N14" s="9"/>
-      <c r="O14" s="9"/>
-      <c r="P14" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M14" s="10">
+        <v>46329.0</v>
+      </c>
+      <c r="N14" s="17">
+        <v>46332.0</v>
+      </c>
+      <c r="O14" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_테스트 계획서_0.01v.docx</v>
       </c>
-      <c r="Q14" s="6"/>
-      <c r="S14" s="14"/>
-      <c r="Y14" s="15"/>
+      <c r="P14" s="6"/>
+      <c r="R14" s="15"/>
+      <c r="X14" s="16"/>
     </row>
     <row r="15" ht="28.5" customHeight="1">
       <c r="B15" s="3" t="s">
+        <v>70</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>67</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>71</v>
+      </c>
+      <c r="E15" s="5" t="s">
         <v>72</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>69</v>
-      </c>
-      <c r="D15" s="5" t="s">
-        <v>73</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>74</v>
-      </c>
       <c r="F15" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G15" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H15" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G15" s="7" t="s">
-        <v>29</v>
-      </c>
-      <c r="H15" s="7" t="s">
-        <v>34</v>
-      </c>
       <c r="I15" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J15" s="3"/>
       <c r="K15" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L15" s="8"/>
-      <c r="M15" s="9"/>
-      <c r="N15" s="9"/>
-      <c r="O15" s="9"/>
-      <c r="P15" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M15" s="10">
+        <v>46329.0</v>
+      </c>
+      <c r="N15" s="17">
+        <v>46343.0</v>
+      </c>
+      <c r="O15" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_테스트 케이스_0.01v.xlsx</v>
       </c>
-      <c r="Q15" s="6"/>
-      <c r="S15" s="14"/>
-      <c r="Y15" s="15"/>
+      <c r="P15" s="6"/>
+      <c r="R15" s="15"/>
+      <c r="X15" s="16"/>
     </row>
     <row r="16" ht="28.5" customHeight="1">
       <c r="B16" s="3" t="s">
+        <v>73</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D16" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="E16" s="5" t="s">
         <v>76</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="F16" s="4" t="s">
         <v>77</v>
       </c>
-      <c r="E16" s="5" t="s">
-        <v>78</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>79</v>
-      </c>
       <c r="G16" s="7" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="I16" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="H16" s="7" t="s">
-        <v>43</v>
-      </c>
-      <c r="I16" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="J16" s="3"/>
       <c r="K16" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L16" s="8"/>
-      <c r="M16" s="9"/>
-      <c r="N16" s="9"/>
-      <c r="O16" s="9"/>
-      <c r="P16" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M16" s="10">
+        <v>46342.0</v>
+      </c>
+      <c r="N16" s="17">
+        <v>46343.0</v>
+      </c>
+      <c r="O16" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_관리자 매뉴얼_0.01v.docx</v>
       </c>
-      <c r="Q16" s="6"/>
-      <c r="S16" s="16"/>
-      <c r="T16" s="17"/>
-      <c r="U16" s="17"/>
-      <c r="V16" s="17"/>
-      <c r="W16" s="17"/>
-      <c r="X16" s="17"/>
-      <c r="Y16" s="18"/>
+      <c r="P16" s="6"/>
+      <c r="R16" s="18"/>
+      <c r="S16" s="19"/>
+      <c r="T16" s="19"/>
+      <c r="U16" s="19"/>
+      <c r="V16" s="19"/>
+      <c r="W16" s="19"/>
+      <c r="X16" s="20"/>
     </row>
     <row r="17" ht="28.5" customHeight="1">
       <c r="B17" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="D17" s="5" t="s">
+        <v>79</v>
+      </c>
+      <c r="E17" s="5" t="s">
         <v>80</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>76</v>
-      </c>
-      <c r="D17" s="5" t="s">
-        <v>81</v>
-      </c>
-      <c r="E17" s="5" t="s">
-        <v>82</v>
-      </c>
       <c r="F17" s="4" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="G17" s="7" t="s">
+        <v>33</v>
+      </c>
+      <c r="H17" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="I17" s="4" t="s">
         <v>34</v>
-      </c>
-      <c r="H17" s="7" t="s">
-        <v>22</v>
-      </c>
-      <c r="I17" s="4" t="s">
-        <v>35</v>
       </c>
       <c r="J17" s="3"/>
       <c r="K17" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L17" s="8"/>
-      <c r="M17" s="9"/>
-      <c r="N17" s="9"/>
-      <c r="O17" s="9"/>
-      <c r="P17" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M17" s="10">
+        <v>46342.0</v>
+      </c>
+      <c r="N17" s="17">
+        <v>46343.0</v>
+      </c>
+      <c r="O17" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_사용자 매뉴얼_0.01v.docx</v>
       </c>
-      <c r="Q17" s="6"/>
+      <c r="P17" s="6"/>
     </row>
     <row r="18" ht="28.5" customHeight="1">
       <c r="B18" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="C18" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D18" s="5" t="s">
+        <v>82</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>83</v>
       </c>
-      <c r="C18" s="4" t="s">
-        <v>31</v>
-      </c>
-      <c r="D18" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>85</v>
-      </c>
       <c r="F18" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="G18" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="G18" s="8"/>
-      <c r="H18" s="8"/>
+      <c r="H18" s="7" t="s">
+        <v>28</v>
+      </c>
       <c r="I18" s="4" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="J18" s="3"/>
       <c r="K18" s="7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="L18" s="8"/>
-      <c r="M18" s="9"/>
-      <c r="N18" s="9"/>
-      <c r="O18" s="9"/>
-      <c r="P18" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="M18" s="10">
+        <v>46323.0</v>
+      </c>
+      <c r="N18" s="21">
+        <v>46325.0</v>
+      </c>
+      <c r="O18" s="6" t="str">
+        <f t="shared" si="1"/>
         <v>Final_Project_기능정의서_0.01v.xlsx</v>
       </c>
-      <c r="Q18" s="6"/>
+      <c r="P18" s="6"/>
     </row>
     <row r="19" ht="28.5" customHeight="1">
       <c r="B19" s="3" t="s">
-        <v>86</v>
-      </c>
-      <c r="C19" s="3"/>
-      <c r="D19" s="5"/>
+        <v>84</v>
+      </c>
+      <c r="C19" s="4" t="s">
+        <v>36</v>
+      </c>
+      <c r="D19" s="5" t="s">
+        <v>85</v>
+      </c>
       <c r="E19" s="6"/>
       <c r="F19" s="3"/>
-      <c r="G19" s="7"/>
-      <c r="H19" s="7"/>
+      <c r="G19" s="7" t="s">
+        <v>21</v>
+      </c>
+      <c r="H19" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="I19" s="3"/>
       <c r="J19" s="3"/>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
-      <c r="M19" s="9"/>
-      <c r="N19" s="9"/>
-      <c r="O19" s="9"/>
-      <c r="P19" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q19" s="6"/>
+      <c r="M19" s="10">
+        <v>46324.0</v>
+      </c>
+      <c r="N19" s="17">
+        <v>46325.0</v>
+      </c>
+      <c r="O19" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project_기술 아키텍처_.</v>
+      </c>
+      <c r="P19" s="6"/>
     </row>
     <row r="20" ht="28.5" customHeight="1">
       <c r="B20" s="3" t="s">
+        <v>86</v>
+      </c>
+      <c r="C20" s="3"/>
+      <c r="D20" s="5" t="s">
         <v>87</v>
       </c>
-      <c r="C20" s="3"/>
-      <c r="D20" s="6"/>
       <c r="E20" s="6"/>
       <c r="F20" s="3"/>
-      <c r="G20" s="7"/>
+      <c r="G20" s="7" t="s">
+        <v>88</v>
+      </c>
       <c r="H20" s="8"/>
       <c r="I20" s="3"/>
       <c r="J20" s="3"/>
       <c r="K20" s="8"/>
       <c r="L20" s="8"/>
-      <c r="M20" s="9"/>
-      <c r="N20" s="9"/>
-      <c r="O20" s="9"/>
-      <c r="P20" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q20" s="6"/>
+      <c r="M20" s="10">
+        <v>46335.0</v>
+      </c>
+      <c r="N20" s="17">
+        <v>46343.0</v>
+      </c>
+      <c r="O20" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project_QA_.</v>
+      </c>
+      <c r="P20" s="6"/>
     </row>
     <row r="21" ht="28.5" customHeight="1">
       <c r="B21" s="3" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C21" s="3"/>
-      <c r="D21" s="6"/>
+      <c r="D21" s="5" t="s">
+        <v>90</v>
+      </c>
       <c r="E21" s="6"/>
       <c r="F21" s="3"/>
-      <c r="G21" s="8"/>
-      <c r="H21" s="8"/>
+      <c r="G21" s="7" t="s">
+        <v>28</v>
+      </c>
+      <c r="H21" s="7" t="s">
+        <v>21</v>
+      </c>
       <c r="I21" s="3"/>
       <c r="J21" s="3"/>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
-      <c r="M21" s="9"/>
-      <c r="N21" s="9"/>
-      <c r="O21" s="9"/>
-      <c r="P21" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q21" s="6"/>
+      <c r="M21" s="10">
+        <v>46328.0</v>
+      </c>
+      <c r="N21" s="17">
+        <v>46332.0</v>
+      </c>
+      <c r="O21" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project_AI 아키텍처_.</v>
+      </c>
+      <c r="P21" s="6"/>
     </row>
     <row r="22" ht="28.5" customHeight="1">
       <c r="B22" s="3" t="s">
-        <v>89</v>
-      </c>
-      <c r="C22" s="3"/>
-      <c r="D22" s="6"/>
-      <c r="E22" s="6"/>
-      <c r="F22" s="3"/>
-      <c r="G22" s="8"/>
+        <v>91</v>
+      </c>
+      <c r="C22" s="4" t="s">
+        <v>92</v>
+      </c>
+      <c r="D22" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="E22" s="5" t="s">
+        <v>94</v>
+      </c>
+      <c r="F22" s="4" t="s">
+        <v>77</v>
+      </c>
+      <c r="G22" s="7" t="s">
+        <v>88</v>
+      </c>
       <c r="H22" s="8"/>
-      <c r="I22" s="3"/>
+      <c r="I22" s="4" t="s">
+        <v>34</v>
+      </c>
       <c r="J22" s="3"/>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
-      <c r="M22" s="9"/>
-      <c r="N22" s="9"/>
-      <c r="O22" s="9"/>
-      <c r="P22" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q22" s="6"/>
+      <c r="M22" s="10">
+        <v>46323.0</v>
+      </c>
+      <c r="N22" s="10">
+        <v>46323.0</v>
+      </c>
+      <c r="O22" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>피드백노트_.docx</v>
+      </c>
+      <c r="P22" s="6"/>
     </row>
     <row r="23" ht="28.5" customHeight="1">
       <c r="B23" s="3" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="C23" s="3"/>
-      <c r="D23" s="6"/>
+      <c r="D23" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E23" s="6"/>
       <c r="F23" s="3"/>
       <c r="G23" s="8"/>
@@ -1724,19 +1864,20 @@
       <c r="L23" s="8"/>
       <c r="M23" s="9"/>
       <c r="N23" s="9"/>
-      <c r="O23" s="9"/>
-      <c r="P23" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q23" s="6"/>
+      <c r="O23" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P23" s="6"/>
     </row>
     <row r="24" ht="28.5" customHeight="1">
       <c r="B24" s="3" t="s">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="C24" s="3"/>
-      <c r="D24" s="6"/>
+      <c r="D24" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E24" s="6"/>
       <c r="F24" s="3"/>
       <c r="G24" s="8"/>
@@ -1747,19 +1888,20 @@
       <c r="L24" s="8"/>
       <c r="M24" s="9"/>
       <c r="N24" s="9"/>
-      <c r="O24" s="9"/>
-      <c r="P24" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q24" s="6"/>
+      <c r="O24" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P24" s="6"/>
     </row>
     <row r="25" ht="28.5" customHeight="1">
       <c r="B25" s="3" t="s">
-        <v>92</v>
+        <v>98</v>
       </c>
       <c r="C25" s="3"/>
-      <c r="D25" s="6"/>
+      <c r="D25" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E25" s="6"/>
       <c r="F25" s="3"/>
       <c r="G25" s="8"/>
@@ -1770,19 +1912,20 @@
       <c r="L25" s="8"/>
       <c r="M25" s="9"/>
       <c r="N25" s="9"/>
-      <c r="O25" s="9"/>
-      <c r="P25" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q25" s="6"/>
+      <c r="O25" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P25" s="6"/>
     </row>
     <row r="26" ht="28.5" customHeight="1">
       <c r="B26" s="3" t="s">
-        <v>93</v>
+        <v>99</v>
       </c>
       <c r="C26" s="3"/>
-      <c r="D26" s="6"/>
+      <c r="D26" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E26" s="6"/>
       <c r="F26" s="3"/>
       <c r="G26" s="8"/>
@@ -1793,19 +1936,20 @@
       <c r="L26" s="8"/>
       <c r="M26" s="9"/>
       <c r="N26" s="9"/>
-      <c r="O26" s="9"/>
-      <c r="P26" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q26" s="6"/>
+      <c r="O26" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P26" s="6"/>
     </row>
     <row r="27" ht="28.5" customHeight="1">
       <c r="B27" s="3" t="s">
-        <v>94</v>
+        <v>100</v>
       </c>
       <c r="C27" s="3"/>
-      <c r="D27" s="6"/>
+      <c r="D27" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E27" s="6"/>
       <c r="F27" s="3"/>
       <c r="G27" s="8"/>
@@ -1816,19 +1960,20 @@
       <c r="L27" s="8"/>
       <c r="M27" s="9"/>
       <c r="N27" s="9"/>
-      <c r="O27" s="9"/>
-      <c r="P27" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q27" s="6"/>
+      <c r="O27" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P27" s="6"/>
     </row>
     <row r="28" ht="28.5" customHeight="1">
       <c r="B28" s="3" t="s">
-        <v>95</v>
+        <v>101</v>
       </c>
       <c r="C28" s="3"/>
-      <c r="D28" s="6"/>
+      <c r="D28" s="5" t="s">
+        <v>96</v>
+      </c>
       <c r="E28" s="6"/>
       <c r="F28" s="3"/>
       <c r="G28" s="8"/>
@@ -1839,16 +1984,15 @@
       <c r="L28" s="8"/>
       <c r="M28" s="9"/>
       <c r="N28" s="9"/>
-      <c r="O28" s="9"/>
-      <c r="P28" s="6" t="str">
-        <f t="shared" si="2"/>
-        <v/>
-      </c>
-      <c r="Q28" s="6"/>
+      <c r="O28" s="6" t="str">
+        <f t="shared" si="1"/>
+        <v>Final_Project__.</v>
+      </c>
+      <c r="P28" s="6"/>
     </row>
     <row r="29" ht="28.5" customHeight="1">
       <c r="B29" s="3" t="s">
-        <v>96</v>
+        <v>102</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="6"/>
@@ -1862,16 +2006,15 @@
       <c r="L29" s="8"/>
       <c r="M29" s="9"/>
       <c r="N29" s="9"/>
-      <c r="O29" s="9"/>
-      <c r="P29" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O29" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q29" s="6"/>
+      <c r="P29" s="6"/>
     </row>
     <row r="30" ht="28.5" customHeight="1">
       <c r="B30" s="3" t="s">
-        <v>97</v>
+        <v>103</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="6"/>
@@ -1885,16 +2028,15 @@
       <c r="L30" s="8"/>
       <c r="M30" s="9"/>
       <c r="N30" s="9"/>
-      <c r="O30" s="9"/>
-      <c r="P30" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O30" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q30" s="6"/>
+      <c r="P30" s="6"/>
     </row>
     <row r="31" ht="28.5" customHeight="1">
       <c r="B31" s="3" t="s">
-        <v>98</v>
+        <v>104</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="6"/>
@@ -1908,16 +2050,15 @@
       <c r="L31" s="8"/>
       <c r="M31" s="9"/>
       <c r="N31" s="9"/>
-      <c r="O31" s="9"/>
-      <c r="P31" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O31" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q31" s="6"/>
+      <c r="P31" s="6"/>
     </row>
     <row r="32" ht="28.5" customHeight="1">
       <c r="B32" s="3" t="s">
-        <v>99</v>
+        <v>105</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="6"/>
@@ -1931,16 +2072,15 @@
       <c r="L32" s="8"/>
       <c r="M32" s="9"/>
       <c r="N32" s="9"/>
-      <c r="O32" s="9"/>
-      <c r="P32" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O32" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q32" s="6"/>
+      <c r="P32" s="6"/>
     </row>
     <row r="33" ht="28.5" customHeight="1">
       <c r="B33" s="3" t="s">
-        <v>100</v>
+        <v>106</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="6"/>
@@ -1954,16 +2094,15 @@
       <c r="L33" s="8"/>
       <c r="M33" s="9"/>
       <c r="N33" s="9"/>
-      <c r="O33" s="9"/>
-      <c r="P33" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O33" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q33" s="6"/>
+      <c r="P33" s="6"/>
     </row>
     <row r="34" ht="28.5" customHeight="1">
       <c r="B34" s="3" t="s">
-        <v>101</v>
+        <v>107</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="6"/>
@@ -1977,16 +2116,15 @@
       <c r="L34" s="8"/>
       <c r="M34" s="9"/>
       <c r="N34" s="9"/>
-      <c r="O34" s="9"/>
-      <c r="P34" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O34" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q34" s="6"/>
+      <c r="P34" s="6"/>
     </row>
     <row r="35" ht="28.5" customHeight="1">
       <c r="B35" s="3" t="s">
-        <v>102</v>
+        <v>108</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="6"/>
@@ -2000,16 +2138,15 @@
       <c r="L35" s="8"/>
       <c r="M35" s="9"/>
       <c r="N35" s="9"/>
-      <c r="O35" s="9"/>
-      <c r="P35" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O35" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q35" s="6"/>
+      <c r="P35" s="6"/>
     </row>
     <row r="36" ht="28.5" customHeight="1">
       <c r="B36" s="3" t="s">
-        <v>103</v>
+        <v>109</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="6"/>
@@ -2023,16 +2160,15 @@
       <c r="L36" s="8"/>
       <c r="M36" s="9"/>
       <c r="N36" s="9"/>
-      <c r="O36" s="9"/>
-      <c r="P36" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O36" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q36" s="6"/>
+      <c r="P36" s="6"/>
     </row>
     <row r="37" ht="28.5" customHeight="1">
       <c r="B37" s="3" t="s">
-        <v>104</v>
+        <v>110</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="6"/>
@@ -2046,16 +2182,15 @@
       <c r="L37" s="8"/>
       <c r="M37" s="9"/>
       <c r="N37" s="9"/>
-      <c r="O37" s="9"/>
-      <c r="P37" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O37" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q37" s="6"/>
+      <c r="P37" s="6"/>
     </row>
     <row r="38" ht="28.5" customHeight="1">
       <c r="B38" s="3" t="s">
-        <v>105</v>
+        <v>111</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="6"/>
@@ -2069,16 +2204,15 @@
       <c r="L38" s="8"/>
       <c r="M38" s="9"/>
       <c r="N38" s="9"/>
-      <c r="O38" s="9"/>
-      <c r="P38" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O38" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q38" s="6"/>
+      <c r="P38" s="6"/>
     </row>
     <row r="39" ht="28.5" customHeight="1">
       <c r="B39" s="3" t="s">
-        <v>106</v>
+        <v>112</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="6"/>
@@ -2092,16 +2226,15 @@
       <c r="L39" s="8"/>
       <c r="M39" s="9"/>
       <c r="N39" s="9"/>
-      <c r="O39" s="9"/>
-      <c r="P39" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O39" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q39" s="6"/>
+      <c r="P39" s="6"/>
     </row>
     <row r="40" ht="28.5" customHeight="1">
       <c r="B40" s="3" t="s">
-        <v>107</v>
+        <v>113</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="6"/>
@@ -2115,16 +2248,15 @@
       <c r="L40" s="8"/>
       <c r="M40" s="9"/>
       <c r="N40" s="9"/>
-      <c r="O40" s="9"/>
-      <c r="P40" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O40" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q40" s="6"/>
+      <c r="P40" s="6"/>
     </row>
     <row r="41" ht="28.5" customHeight="1">
       <c r="B41" s="3" t="s">
-        <v>108</v>
+        <v>114</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="6"/>
@@ -2138,16 +2270,15 @@
       <c r="L41" s="8"/>
       <c r="M41" s="9"/>
       <c r="N41" s="9"/>
-      <c r="O41" s="9"/>
-      <c r="P41" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O41" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q41" s="6"/>
+      <c r="P41" s="6"/>
     </row>
     <row r="42" ht="28.5" customHeight="1">
       <c r="B42" s="3" t="s">
-        <v>109</v>
+        <v>115</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="6"/>
@@ -2161,16 +2292,15 @@
       <c r="L42" s="8"/>
       <c r="M42" s="9"/>
       <c r="N42" s="9"/>
-      <c r="O42" s="9"/>
-      <c r="P42" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O42" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q42" s="6"/>
+      <c r="P42" s="6"/>
     </row>
     <row r="43" ht="28.5" customHeight="1">
       <c r="B43" s="3" t="s">
-        <v>110</v>
+        <v>116</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="6"/>
@@ -2184,16 +2314,15 @@
       <c r="L43" s="8"/>
       <c r="M43" s="9"/>
       <c r="N43" s="9"/>
-      <c r="O43" s="9"/>
-      <c r="P43" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O43" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q43" s="6"/>
+      <c r="P43" s="6"/>
     </row>
     <row r="44" ht="28.5" customHeight="1">
       <c r="B44" s="3" t="s">
-        <v>111</v>
+        <v>117</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="6"/>
@@ -2207,16 +2336,15 @@
       <c r="L44" s="8"/>
       <c r="M44" s="9"/>
       <c r="N44" s="9"/>
-      <c r="O44" s="9"/>
-      <c r="P44" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O44" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q44" s="6"/>
+      <c r="P44" s="6"/>
     </row>
     <row r="45" ht="28.5" customHeight="1">
       <c r="B45" s="3" t="s">
-        <v>112</v>
+        <v>118</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="6"/>
@@ -2230,16 +2358,15 @@
       <c r="L45" s="8"/>
       <c r="M45" s="9"/>
       <c r="N45" s="9"/>
-      <c r="O45" s="9"/>
-      <c r="P45" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O45" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q45" s="6"/>
+      <c r="P45" s="6"/>
     </row>
     <row r="46" ht="28.5" customHeight="1">
       <c r="B46" s="3" t="s">
-        <v>113</v>
+        <v>119</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="6"/>
@@ -2253,16 +2380,15 @@
       <c r="L46" s="8"/>
       <c r="M46" s="9"/>
       <c r="N46" s="9"/>
-      <c r="O46" s="9"/>
-      <c r="P46" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O46" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q46" s="6"/>
+      <c r="P46" s="6"/>
     </row>
     <row r="47" ht="28.5" customHeight="1">
       <c r="B47" s="3" t="s">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="6"/>
@@ -2276,16 +2402,15 @@
       <c r="L47" s="8"/>
       <c r="M47" s="9"/>
       <c r="N47" s="9"/>
-      <c r="O47" s="9"/>
-      <c r="P47" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O47" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q47" s="6"/>
+      <c r="P47" s="6"/>
     </row>
     <row r="48" ht="28.5" customHeight="1">
       <c r="B48" s="3" t="s">
-        <v>115</v>
+        <v>121</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="6"/>
@@ -2299,16 +2424,15 @@
       <c r="L48" s="8"/>
       <c r="M48" s="9"/>
       <c r="N48" s="9"/>
-      <c r="O48" s="9"/>
-      <c r="P48" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O48" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q48" s="6"/>
+      <c r="P48" s="6"/>
     </row>
     <row r="49" ht="28.5" customHeight="1">
       <c r="B49" s="3" t="s">
-        <v>116</v>
+        <v>122</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="6"/>
@@ -2322,16 +2446,15 @@
       <c r="L49" s="8"/>
       <c r="M49" s="9"/>
       <c r="N49" s="9"/>
-      <c r="O49" s="9"/>
-      <c r="P49" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O49" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q49" s="6"/>
+      <c r="P49" s="6"/>
     </row>
     <row r="50" ht="28.5" customHeight="1">
       <c r="B50" s="3" t="s">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="6"/>
@@ -2345,16 +2468,15 @@
       <c r="L50" s="8"/>
       <c r="M50" s="9"/>
       <c r="N50" s="9"/>
-      <c r="O50" s="9"/>
-      <c r="P50" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O50" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q50" s="6"/>
+      <c r="P50" s="6"/>
     </row>
     <row r="51" ht="28.5" customHeight="1">
       <c r="B51" s="3" t="s">
-        <v>118</v>
+        <v>124</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="6"/>
@@ -2368,16 +2490,15 @@
       <c r="L51" s="8"/>
       <c r="M51" s="9"/>
       <c r="N51" s="9"/>
-      <c r="O51" s="9"/>
-      <c r="P51" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O51" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q51" s="6"/>
+      <c r="P51" s="6"/>
     </row>
     <row r="52" ht="28.5" customHeight="1">
       <c r="B52" s="3" t="s">
-        <v>119</v>
+        <v>125</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="6"/>
@@ -2391,16 +2512,15 @@
       <c r="L52" s="8"/>
       <c r="M52" s="9"/>
       <c r="N52" s="9"/>
-      <c r="O52" s="9"/>
-      <c r="P52" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O52" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q52" s="6"/>
+      <c r="P52" s="6"/>
     </row>
     <row r="53" ht="28.5" customHeight="1">
       <c r="B53" s="3" t="s">
-        <v>120</v>
+        <v>126</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="6"/>
@@ -2414,16 +2534,15 @@
       <c r="L53" s="8"/>
       <c r="M53" s="9"/>
       <c r="N53" s="9"/>
-      <c r="O53" s="9"/>
-      <c r="P53" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O53" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q53" s="6"/>
+      <c r="P53" s="6"/>
     </row>
     <row r="54" ht="28.5" customHeight="1">
       <c r="B54" s="3" t="s">
-        <v>121</v>
+        <v>127</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="6"/>
@@ -2437,16 +2556,15 @@
       <c r="L54" s="8"/>
       <c r="M54" s="9"/>
       <c r="N54" s="9"/>
-      <c r="O54" s="9"/>
-      <c r="P54" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O54" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q54" s="6"/>
+      <c r="P54" s="6"/>
     </row>
     <row r="55" ht="28.5" customHeight="1">
       <c r="B55" s="3" t="s">
-        <v>122</v>
+        <v>128</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="6"/>
@@ -2460,16 +2578,15 @@
       <c r="L55" s="8"/>
       <c r="M55" s="9"/>
       <c r="N55" s="9"/>
-      <c r="O55" s="9"/>
-      <c r="P55" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O55" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q55" s="6"/>
+      <c r="P55" s="6"/>
     </row>
     <row r="56" ht="28.5" customHeight="1">
       <c r="B56" s="3" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="6"/>
@@ -2483,16 +2600,15 @@
       <c r="L56" s="8"/>
       <c r="M56" s="9"/>
       <c r="N56" s="9"/>
-      <c r="O56" s="9"/>
-      <c r="P56" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O56" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q56" s="6"/>
+      <c r="P56" s="6"/>
     </row>
     <row r="57" ht="28.5" customHeight="1">
       <c r="B57" s="3" t="s">
-        <v>124</v>
+        <v>130</v>
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="6"/>
@@ -2506,16 +2622,15 @@
       <c r="L57" s="8"/>
       <c r="M57" s="9"/>
       <c r="N57" s="9"/>
-      <c r="O57" s="9"/>
-      <c r="P57" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O57" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q57" s="6"/>
+      <c r="P57" s="6"/>
     </row>
     <row r="58" ht="28.5" customHeight="1">
       <c r="B58" s="3" t="s">
-        <v>125</v>
+        <v>131</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="6"/>
@@ -2529,16 +2644,15 @@
       <c r="L58" s="8"/>
       <c r="M58" s="9"/>
       <c r="N58" s="9"/>
-      <c r="O58" s="9"/>
-      <c r="P58" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O58" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q58" s="6"/>
+      <c r="P58" s="6"/>
     </row>
     <row r="59" ht="28.5" customHeight="1">
       <c r="B59" s="3" t="s">
-        <v>126</v>
+        <v>132</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="6"/>
@@ -2552,16 +2666,15 @@
       <c r="L59" s="8"/>
       <c r="M59" s="9"/>
       <c r="N59" s="9"/>
-      <c r="O59" s="9"/>
-      <c r="P59" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O59" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q59" s="6"/>
+      <c r="P59" s="6"/>
     </row>
     <row r="60" ht="28.5" customHeight="1">
       <c r="B60" s="3" t="s">
-        <v>127</v>
+        <v>133</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="6"/>
@@ -2575,12 +2688,11 @@
       <c r="L60" s="8"/>
       <c r="M60" s="9"/>
       <c r="N60" s="9"/>
-      <c r="O60" s="9"/>
-      <c r="P60" s="6" t="str">
-        <f t="shared" si="2"/>
+      <c r="O60" s="6" t="str">
+        <f t="shared" si="1"/>
         <v/>
       </c>
-      <c r="Q60" s="6"/>
+      <c r="P60" s="6"/>
     </row>
     <row r="61" ht="16.5" customHeight="1"/>
     <row r="62" ht="16.5" customHeight="1"/>
@@ -3523,9 +3635,9 @@
     <row r="999" ht="16.5" customHeight="1"/>
     <row r="1000" ht="16.5" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$B$2:$Q$60"/>
+  <autoFilter ref="$B$2:$P$60"/>
   <mergeCells count="1">
-    <mergeCell ref="S4:Y4"/>
+    <mergeCell ref="R4:X16"/>
   </mergeCells>
   <conditionalFormatting sqref="J3:J60">
     <cfRule type="expression" dxfId="0" priority="1">
@@ -3547,9 +3659,9 @@
       <formula>$J3="폐기"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="O3:O60">
+  <conditionalFormatting sqref="N3:N60">
     <cfRule type="expression" dxfId="4" priority="5">
-      <formula>AND($O3&lt;&gt;"",$O3&lt;TODAY(),$J3&lt;&gt;"완료",$J3&lt;&gt;"폐기")</formula>
+      <formula>AND($N3&lt;&gt;"",$N3&lt;TODAY(),$J3&lt;&gt;"완료",$J3&lt;&gt;"폐기")</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations>

</xml_diff>

<commit_message>
update PRD, flowchart upload TRD, displaydecription,
</commit_message>
<xml_diff>
--- a/Final_Project_파일_관리_대장.xlsx
+++ b/Final_Project_파일_관리_대장.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="134">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="133">
   <si>
     <t>No.</t>
   </si>
@@ -165,7 +165,7 @@
     <t>혜현</t>
   </si>
   <si>
-    <t>pptx</t>
+    <t>md</t>
   </si>
   <si>
     <t>05</t>
@@ -176,9 +176,6 @@
   <si>
     <t>AI 면접 프로그램에 대한 플로우 차트. 전체적인 흐름을
 도식화해서 표현함.</t>
-  </si>
-  <si>
-    <t>md</t>
   </si>
   <si>
     <t>검토중</t>
@@ -1170,8 +1167,8 @@
       <c r="M6" s="10">
         <v>46323.0</v>
       </c>
-      <c r="N6" s="17">
-        <v>46325.0</v>
+      <c r="N6" s="14">
+        <v>46323.0</v>
       </c>
       <c r="O6" s="6" t="str">
         <f t="shared" si="1"/>
@@ -1214,12 +1211,12 @@
       <c r="M7" s="10">
         <v>46322.0</v>
       </c>
-      <c r="N7" s="17">
-        <v>46325.0</v>
+      <c r="N7" s="14">
+        <v>46323.0</v>
       </c>
       <c r="O7" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_화면정의서_0.01v.pptx</v>
+        <v>Final_Project_화면정의서_0.01v.md</v>
       </c>
       <c r="P7" s="6"/>
       <c r="R7" s="15"/>
@@ -1248,10 +1245,10 @@
         <v>21</v>
       </c>
       <c r="I8" s="4" t="s">
+        <v>43</v>
+      </c>
+      <c r="J8" s="4" t="s">
         <v>47</v>
-      </c>
-      <c r="J8" s="4" t="s">
-        <v>48</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>24</v>
@@ -1273,16 +1270,16 @@
     </row>
     <row r="9">
       <c r="B9" s="3" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C9" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D9" s="5" t="s">
+        <v>49</v>
+      </c>
+      <c r="E9" s="5" t="s">
         <v>50</v>
-      </c>
-      <c r="E9" s="5" t="s">
-        <v>51</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>19</v>
@@ -1294,7 +1291,7 @@
         <v>21</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="J9" s="3"/>
       <c r="K9" s="7" t="s">
@@ -1317,16 +1314,16 @@
     </row>
     <row r="10" ht="28.5" customHeight="1">
       <c r="B10" s="3" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E10" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>19</v>
@@ -1338,9 +1335,11 @@
         <v>21</v>
       </c>
       <c r="I10" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="J10" s="3"/>
+        <v>34</v>
+      </c>
+      <c r="J10" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="K10" s="7" t="s">
         <v>24</v>
       </c>
@@ -1353,7 +1352,7 @@
       </c>
       <c r="O10" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_시나리오 기획서_0.01v.xlsx</v>
+        <v>Final_Project_시나리오 기획서_0.01v.docx</v>
       </c>
       <c r="P10" s="6"/>
       <c r="R10" s="15"/>
@@ -1361,16 +1360,16 @@
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="5" t="s">
+        <v>56</v>
+      </c>
+      <c r="E11" s="5" t="s">
         <v>57</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>58</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>19</v>
@@ -1405,16 +1404,16 @@
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="B12" s="3" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C12" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>59</v>
+      </c>
+      <c r="E12" s="5" t="s">
         <v>60</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>61</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>19</v>
@@ -1426,7 +1425,7 @@
         <v>33</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="J12" s="3"/>
       <c r="K12" s="7" t="s">
@@ -1449,16 +1448,16 @@
     </row>
     <row r="13" ht="28.5" customHeight="1">
       <c r="B13" s="3" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C13" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="E13" s="5" t="s">
         <v>64</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>65</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>19</v>
@@ -1493,16 +1492,16 @@
     </row>
     <row r="14" ht="28.5" customHeight="1">
       <c r="B14" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="C14" s="4" t="s">
         <v>66</v>
       </c>
-      <c r="C14" s="4" t="s">
+      <c r="D14" s="5" t="s">
         <v>67</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="E14" s="5" t="s">
         <v>68</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>69</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>19</v>
@@ -1537,16 +1536,16 @@
     </row>
     <row r="15" ht="28.5" customHeight="1">
       <c r="B15" s="3" t="s">
+        <v>69</v>
+      </c>
+      <c r="C15" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D15" s="5" t="s">
         <v>70</v>
       </c>
-      <c r="C15" s="4" t="s">
-        <v>67</v>
-      </c>
-      <c r="D15" s="5" t="s">
+      <c r="E15" s="5" t="s">
         <v>71</v>
-      </c>
-      <c r="E15" s="5" t="s">
-        <v>72</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>19</v>
@@ -1581,19 +1580,19 @@
     </row>
     <row r="16" ht="28.5" customHeight="1">
       <c r="B16" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="C16" s="4" t="s">
         <v>73</v>
       </c>
-      <c r="C16" s="4" t="s">
+      <c r="D16" s="5" t="s">
         <v>74</v>
       </c>
-      <c r="D16" s="5" t="s">
+      <c r="E16" s="5" t="s">
         <v>75</v>
       </c>
-      <c r="E16" s="5" t="s">
+      <c r="F16" s="4" t="s">
         <v>76</v>
-      </c>
-      <c r="F16" s="4" t="s">
-        <v>77</v>
       </c>
       <c r="G16" s="7" t="s">
         <v>42</v>
@@ -1630,19 +1629,19 @@
     </row>
     <row r="17" ht="28.5" customHeight="1">
       <c r="B17" s="3" t="s">
+        <v>77</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>73</v>
+      </c>
+      <c r="D17" s="5" t="s">
         <v>78</v>
       </c>
-      <c r="C17" s="4" t="s">
-        <v>74</v>
-      </c>
-      <c r="D17" s="5" t="s">
+      <c r="E17" s="5" t="s">
         <v>79</v>
       </c>
-      <c r="E17" s="5" t="s">
-        <v>80</v>
-      </c>
       <c r="F17" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>33</v>
@@ -1672,16 +1671,16 @@
     </row>
     <row r="18" ht="28.5" customHeight="1">
       <c r="B18" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="5" t="s">
+        <v>81</v>
+      </c>
+      <c r="E18" s="5" t="s">
         <v>82</v>
-      </c>
-      <c r="E18" s="5" t="s">
-        <v>83</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>19</v>
@@ -1714,13 +1713,13 @@
     </row>
     <row r="19" ht="28.5" customHeight="1">
       <c r="B19" s="3" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C19" s="4" t="s">
         <v>36</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="E19" s="6"/>
       <c r="F19" s="3"/>
@@ -1748,16 +1747,16 @@
     </row>
     <row r="20" ht="28.5" customHeight="1">
       <c r="B20" s="3" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C20" s="3"/>
       <c r="D20" s="5" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="E20" s="6"/>
       <c r="F20" s="3"/>
       <c r="G20" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="3"/>
@@ -1778,11 +1777,11 @@
     </row>
     <row r="21" ht="28.5" customHeight="1">
       <c r="B21" s="3" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C21" s="3"/>
       <c r="D21" s="5" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="E21" s="6"/>
       <c r="F21" s="3"/>
@@ -1810,22 +1809,22 @@
     </row>
     <row r="22" ht="28.5" customHeight="1">
       <c r="B22" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="C22" s="4" t="s">
         <v>91</v>
       </c>
-      <c r="C22" s="4" t="s">
+      <c r="D22" s="5" t="s">
         <v>92</v>
       </c>
-      <c r="D22" s="5" t="s">
+      <c r="E22" s="5" t="s">
         <v>93</v>
       </c>
-      <c r="E22" s="5" t="s">
-        <v>94</v>
-      </c>
       <c r="F22" s="4" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="4" t="s">
@@ -1848,11 +1847,11 @@
     </row>
     <row r="23" ht="28.5" customHeight="1">
       <c r="B23" s="3" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="3"/>
@@ -1872,11 +1871,11 @@
     </row>
     <row r="24" ht="28.5" customHeight="1">
       <c r="B24" s="3" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="3"/>
@@ -1896,11 +1895,11 @@
     </row>
     <row r="25" ht="28.5" customHeight="1">
       <c r="B25" s="3" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="3"/>
@@ -1920,11 +1919,11 @@
     </row>
     <row r="26" ht="28.5" customHeight="1">
       <c r="B26" s="3" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="3"/>
@@ -1944,11 +1943,11 @@
     </row>
     <row r="27" ht="28.5" customHeight="1">
       <c r="B27" s="3" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="3"/>
@@ -1968,11 +1967,11 @@
     </row>
     <row r="28" ht="28.5" customHeight="1">
       <c r="B28" s="3" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="5" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="3"/>
@@ -1992,7 +1991,7 @@
     </row>
     <row r="29" ht="28.5" customHeight="1">
       <c r="B29" s="3" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="6"/>
@@ -2014,7 +2013,7 @@
     </row>
     <row r="30" ht="28.5" customHeight="1">
       <c r="B30" s="3" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="6"/>
@@ -2036,7 +2035,7 @@
     </row>
     <row r="31" ht="28.5" customHeight="1">
       <c r="B31" s="3" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="6"/>
@@ -2058,7 +2057,7 @@
     </row>
     <row r="32" ht="28.5" customHeight="1">
       <c r="B32" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="6"/>
@@ -2080,7 +2079,7 @@
     </row>
     <row r="33" ht="28.5" customHeight="1">
       <c r="B33" s="3" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="6"/>
@@ -2102,7 +2101,7 @@
     </row>
     <row r="34" ht="28.5" customHeight="1">
       <c r="B34" s="3" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="6"/>
@@ -2124,7 +2123,7 @@
     </row>
     <row r="35" ht="28.5" customHeight="1">
       <c r="B35" s="3" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="6"/>
@@ -2146,7 +2145,7 @@
     </row>
     <row r="36" ht="28.5" customHeight="1">
       <c r="B36" s="3" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="6"/>
@@ -2168,7 +2167,7 @@
     </row>
     <row r="37" ht="28.5" customHeight="1">
       <c r="B37" s="3" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="6"/>
@@ -2190,7 +2189,7 @@
     </row>
     <row r="38" ht="28.5" customHeight="1">
       <c r="B38" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="6"/>
@@ -2212,7 +2211,7 @@
     </row>
     <row r="39" ht="28.5" customHeight="1">
       <c r="B39" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="6"/>
@@ -2234,7 +2233,7 @@
     </row>
     <row r="40" ht="28.5" customHeight="1">
       <c r="B40" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="6"/>
@@ -2256,7 +2255,7 @@
     </row>
     <row r="41" ht="28.5" customHeight="1">
       <c r="B41" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="6"/>
@@ -2278,7 +2277,7 @@
     </row>
     <row r="42" ht="28.5" customHeight="1">
       <c r="B42" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="6"/>
@@ -2300,7 +2299,7 @@
     </row>
     <row r="43" ht="28.5" customHeight="1">
       <c r="B43" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="6"/>
@@ -2322,7 +2321,7 @@
     </row>
     <row r="44" ht="28.5" customHeight="1">
       <c r="B44" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="6"/>
@@ -2344,7 +2343,7 @@
     </row>
     <row r="45" ht="28.5" customHeight="1">
       <c r="B45" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="6"/>
@@ -2366,7 +2365,7 @@
     </row>
     <row r="46" ht="28.5" customHeight="1">
       <c r="B46" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="6"/>
@@ -2388,7 +2387,7 @@
     </row>
     <row r="47" ht="28.5" customHeight="1">
       <c r="B47" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="6"/>
@@ -2410,7 +2409,7 @@
     </row>
     <row r="48" ht="28.5" customHeight="1">
       <c r="B48" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="6"/>
@@ -2432,7 +2431,7 @@
     </row>
     <row r="49" ht="28.5" customHeight="1">
       <c r="B49" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="6"/>
@@ -2454,7 +2453,7 @@
     </row>
     <row r="50" ht="28.5" customHeight="1">
       <c r="B50" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="6"/>
@@ -2476,7 +2475,7 @@
     </row>
     <row r="51" ht="28.5" customHeight="1">
       <c r="B51" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="6"/>
@@ -2498,7 +2497,7 @@
     </row>
     <row r="52" ht="28.5" customHeight="1">
       <c r="B52" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="6"/>
@@ -2520,7 +2519,7 @@
     </row>
     <row r="53" ht="28.5" customHeight="1">
       <c r="B53" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="6"/>
@@ -2542,7 +2541,7 @@
     </row>
     <row r="54" ht="28.5" customHeight="1">
       <c r="B54" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="6"/>
@@ -2564,7 +2563,7 @@
     </row>
     <row r="55" ht="28.5" customHeight="1">
       <c r="B55" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="6"/>
@@ -2586,7 +2585,7 @@
     </row>
     <row r="56" ht="28.5" customHeight="1">
       <c r="B56" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="6"/>
@@ -2608,7 +2607,7 @@
     </row>
     <row r="57" ht="28.5" customHeight="1">
       <c r="B57" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="6"/>
@@ -2630,7 +2629,7 @@
     </row>
     <row r="58" ht="28.5" customHeight="1">
       <c r="B58" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="6"/>
@@ -2652,7 +2651,7 @@
     </row>
     <row r="59" ht="28.5" customHeight="1">
       <c r="B59" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="6"/>
@@ -2674,7 +2673,7 @@
     </row>
     <row r="60" ht="28.5" customHeight="1">
       <c r="B60" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="6"/>

</xml_diff>

<commit_message>
update file list, WBS
</commit_message>
<xml_diff>
--- a/Final_Project_파일_관리_대장.xlsx
+++ b/Final_Project_파일_관리_대장.xlsx
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="229" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="247" uniqueCount="142">
   <si>
     <t>No.</t>
   </si>
@@ -141,6 +141,12 @@
     <t>docx</t>
   </si>
   <si>
+    <t>완료</t>
+  </si>
+  <si>
+    <t>1.3v</t>
+  </si>
+  <si>
     <t>04</t>
   </si>
   <si>
@@ -153,6 +159,12 @@
     <t>서비스의 기술 구조, 개발 스택, 데이터 흐름 및 시스템 아키텍처를 정의한 기술 문서</t>
   </si>
   <si>
+    <t>검토중</t>
+  </si>
+  <si>
+    <t>1.1v</t>
+  </si>
+  <si>
     <t>10</t>
   </si>
   <si>
@@ -166,6 +178,9 @@
   </si>
   <si>
     <t>md</t>
+  </si>
+  <si>
+    <t>0.3v</t>
   </si>
   <si>
     <t>05</t>
@@ -178,7 +193,7 @@
 도식화해서 표현함.</t>
   </si>
   <si>
-    <t>검토중</t>
+    <t>08v</t>
   </si>
   <si>
     <t>06</t>
@@ -190,9 +205,6 @@
     <t>프론트엔드와 백엔드, 또는 외부 시스템 간에 '어떤 방식으로 데이터를 주고받을 것인가'를 약속한 데이터 규격서</t>
   </si>
   <si>
-    <t>yaml</t>
-  </si>
-  <si>
     <t>07</t>
   </si>
   <si>
@@ -223,6 +235,9 @@
     <t>png</t>
   </si>
   <si>
+    <t>작성전</t>
+  </si>
+  <si>
     <t>11</t>
   </si>
   <si>
@@ -232,6 +247,9 @@
     <t>데이터베이스의 테이블·컬럼·자료형·제약조건·키 관계를 항목별로 기술한 설계 문서</t>
   </si>
   <si>
+    <t>원래는 테이블정의서와 ERD를 분리해야함.  지금은 ERD와 통합</t>
+  </si>
+  <si>
     <t>12</t>
   </si>
   <si>
@@ -292,12 +310,18 @@
     <t>Final_Project_기술 아키텍처</t>
   </si>
   <si>
+    <t>프로젝트의 전체 시스템 구조와 기술 스택, 프론트엔드·백엔드·데이터베이스 간 연동 방식, 서버 구성 및 데이터 흐름을 정의하는 문서입니다.</t>
+  </si>
+  <si>
     <t>18</t>
   </si>
   <si>
     <t>Final_Project_QA</t>
   </si>
   <si>
+    <t>프로젝트 개발 및 검토 과정에서 발생하는 질문, 문제점, 개선 의견과 답변을 기록하고, 해결 여부 및 후속 조치 사항을 관리하는 문서입니다.</t>
+  </si>
+  <si>
     <t>전체</t>
   </si>
   <si>
@@ -305,6 +329,9 @@
   </si>
   <si>
     <t>Final_Project_AI 아키텍처</t>
+  </si>
+  <si>
+    <t>AI 면접 시스템에 적용되는 LLM, RAG, STT, TTS, 영상·음성 분석 등 AI 기술의 구성과 모델별 역할, 데이터 처리 과정 및 AI 기능 간 연동 구조를 정의하는 문서입니다.</t>
   </si>
   <si>
     <t>20</t>
@@ -443,7 +470,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="yyyy\-mm\-dd"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="7">
     <font>
       <sz val="11.0"/>
       <color theme="1"/>
@@ -473,19 +500,8 @@
     </font>
     <font/>
     <font>
-      <b/>
-      <sz val="11.0"/>
-      <color rgb="FFFF0000"/>
-      <name val="Noto Sans KR"/>
-    </font>
-    <font>
       <sz val="11.0"/>
       <color rgb="FFF79646"/>
-      <name val="Noto Sans KR"/>
-    </font>
-    <font>
-      <sz val="11.0"/>
-      <color theme="9"/>
       <name val="Noto Sans KR"/>
     </font>
   </fonts>
@@ -575,7 +591,7 @@
   <cellStyleXfs count="1">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
       <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
     </xf>
@@ -612,20 +628,14 @@
     <xf borderId="2" fillId="0" fontId="4" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="3" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="4" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
     <xf borderId="5" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="6" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="7" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="1" fillId="0" fontId="6" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
       <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
     </xf>
     <xf borderId="7" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="8" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
     <xf borderId="9" fillId="0" fontId="5" numFmtId="0" xfId="0" applyBorder="1" applyFont="1"/>
-    <xf borderId="1" fillId="0" fontId="8" numFmtId="164" xfId="0" applyAlignment="1" applyBorder="1" applyFont="1" applyNumberFormat="1">
-      <alignment horizontal="center" readingOrder="0" shrinkToFit="0" vertical="center" wrapText="1"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle xfId="0" name="Normal" builtinId="0"/>
@@ -1111,39 +1121,41 @@
       <c r="I5" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="J5" s="3" t="s">
-        <v>23</v>
+      <c r="J5" s="4" t="s">
+        <v>35</v>
       </c>
       <c r="K5" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="8"/>
+      <c r="L5" s="7" t="s">
+        <v>36</v>
+      </c>
       <c r="M5" s="10">
         <v>46322.0</v>
       </c>
-      <c r="N5" s="14">
+      <c r="N5" s="10">
         <v>46323.0</v>
       </c>
       <c r="O5" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_PRD정의서_0.01v.docx</v>
+        <v>Final_Project_PRD정의서_1.3v.docx</v>
       </c>
       <c r="P5" s="6"/>
-      <c r="R5" s="15"/>
-      <c r="X5" s="16"/>
+      <c r="R5" s="14"/>
+      <c r="X5" s="15"/>
     </row>
     <row r="6" ht="28.5" customHeight="1">
       <c r="B6" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F6" s="3" t="s">
         <v>19</v>
@@ -1157,39 +1169,41 @@
       <c r="I6" s="3" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="3" t="s">
-        <v>23</v>
+      <c r="J6" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="K6" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L6" s="8"/>
+      <c r="L6" s="7" t="s">
+        <v>42</v>
+      </c>
       <c r="M6" s="10">
         <v>46323.0</v>
       </c>
-      <c r="N6" s="14">
+      <c r="N6" s="10">
         <v>46323.0</v>
       </c>
       <c r="O6" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_TRD정의서_0.01v.docx</v>
+        <v>Final_Project_TRD정의서_1.1v.docx</v>
       </c>
       <c r="P6" s="6"/>
-      <c r="R6" s="15"/>
-      <c r="X6" s="16"/>
+      <c r="R6" s="14"/>
+      <c r="X6" s="15"/>
     </row>
     <row r="7">
       <c r="B7" s="3" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="C7" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="E7" s="5" t="s">
-        <v>41</v>
+        <v>45</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>19</v>
@@ -1198,62 +1212,68 @@
         <v>21</v>
       </c>
       <c r="H7" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I7" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="J7" s="3"/>
+        <v>47</v>
+      </c>
+      <c r="J7" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="K7" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L7" s="8"/>
+      <c r="L7" s="7" t="s">
+        <v>48</v>
+      </c>
       <c r="M7" s="10">
         <v>46322.0</v>
       </c>
-      <c r="N7" s="14">
+      <c r="N7" s="10">
         <v>46323.0</v>
       </c>
       <c r="O7" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_화면정의서_0.01v.md</v>
+        <v>Final_Project_화면정의서_0.3v.md</v>
       </c>
       <c r="P7" s="6"/>
-      <c r="R7" s="15"/>
-      <c r="X7" s="16"/>
+      <c r="R7" s="14"/>
+      <c r="X7" s="15"/>
     </row>
     <row r="8" ht="28.5" customHeight="1">
       <c r="B8" s="3" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="C8" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="E8" s="5" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="F8" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G8" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H8" s="7" t="s">
         <v>21</v>
       </c>
       <c r="I8" s="4" t="s">
-        <v>43</v>
+        <v>47</v>
       </c>
       <c r="J8" s="4" t="s">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="K8" s="7" t="s">
         <v>24</v>
       </c>
-      <c r="L8" s="8"/>
+      <c r="L8" s="7" t="s">
+        <v>52</v>
+      </c>
       <c r="M8" s="10">
         <v>46317.0</v>
       </c>
@@ -1262,38 +1282,40 @@
       </c>
       <c r="O8" s="5" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_서비스 플로우차트_0.01v.md</v>
+        <v>Final_Project_서비스 플로우차트_08v.md</v>
       </c>
       <c r="P8" s="6"/>
-      <c r="R8" s="15"/>
-      <c r="X8" s="16"/>
+      <c r="R8" s="14"/>
+      <c r="X8" s="15"/>
     </row>
     <row r="9">
       <c r="B9" s="3" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="C9" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="E9" s="5" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="F9" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G9" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H9" s="7" t="s">
         <v>21</v>
       </c>
       <c r="I9" s="4" t="s">
-        <v>51</v>
-      </c>
-      <c r="J9" s="3"/>
+        <v>47</v>
+      </c>
+      <c r="J9" s="4" t="s">
+        <v>41</v>
+      </c>
       <c r="K9" s="7" t="s">
         <v>24</v>
       </c>
@@ -1301,35 +1323,35 @@
       <c r="M9" s="10">
         <v>46325.0</v>
       </c>
-      <c r="N9" s="17">
+      <c r="N9" s="16">
         <v>46332.0</v>
       </c>
       <c r="O9" s="6" t="str">
         <f t="shared" si="1"/>
-        <v>Final_Project_API 명세서_0.01v.yaml</v>
+        <v>Final_Project_API 명세서_0.01v.md</v>
       </c>
       <c r="P9" s="6"/>
-      <c r="R9" s="15"/>
-      <c r="X9" s="16"/>
+      <c r="R9" s="14"/>
+      <c r="X9" s="15"/>
     </row>
     <row r="10" ht="28.5" customHeight="1">
       <c r="B10" s="3" t="s">
-        <v>52</v>
+        <v>56</v>
       </c>
       <c r="C10" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>53</v>
+        <v>57</v>
       </c>
       <c r="E10" s="5" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="F10" s="4" t="s">
         <v>19</v>
       </c>
       <c r="G10" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H10" s="7" t="s">
         <v>21</v>
@@ -1338,7 +1360,7 @@
         <v>34</v>
       </c>
       <c r="J10" s="4" t="s">
-        <v>23</v>
+        <v>35</v>
       </c>
       <c r="K10" s="7" t="s">
         <v>24</v>
@@ -1347,29 +1369,29 @@
       <c r="M10" s="10">
         <v>46323.0</v>
       </c>
-      <c r="N10" s="17">
-        <v>46325.0</v>
+      <c r="N10" s="10">
+        <v>46324.0</v>
       </c>
       <c r="O10" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_시나리오 기획서_0.01v.docx</v>
       </c>
       <c r="P10" s="6"/>
-      <c r="R10" s="15"/>
-      <c r="X10" s="16"/>
+      <c r="R10" s="14"/>
+      <c r="X10" s="15"/>
     </row>
     <row r="11">
       <c r="B11" s="3" t="s">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="C11" s="4" t="s">
         <v>16</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="E11" s="5" t="s">
-        <v>57</v>
+        <v>61</v>
       </c>
       <c r="F11" s="4" t="s">
         <v>19</v>
@@ -1399,21 +1421,21 @@
         <v>Final_Project_WBS_업무관리_0.01v.xlsx</v>
       </c>
       <c r="P11" s="6"/>
-      <c r="R11" s="15"/>
-      <c r="X11" s="16"/>
+      <c r="R11" s="14"/>
+      <c r="X11" s="15"/>
     </row>
     <row r="12" ht="28.5" customHeight="1">
       <c r="B12" s="3" t="s">
-        <v>58</v>
+        <v>62</v>
       </c>
       <c r="C12" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>59</v>
+        <v>63</v>
       </c>
       <c r="E12" s="5" t="s">
-        <v>60</v>
+        <v>64</v>
       </c>
       <c r="F12" s="4" t="s">
         <v>19</v>
@@ -1425,39 +1447,41 @@
         <v>33</v>
       </c>
       <c r="I12" s="4" t="s">
-        <v>61</v>
-      </c>
-      <c r="J12" s="3"/>
+        <v>65</v>
+      </c>
+      <c r="J12" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="K12" s="7" t="s">
         <v>24</v>
       </c>
       <c r="L12" s="8"/>
       <c r="M12" s="10">
-        <v>46325.0</v>
-      </c>
-      <c r="N12" s="17">
-        <v>46332.0</v>
+        <v>46324.0</v>
+      </c>
+      <c r="N12" s="10">
+        <v>46324.0</v>
       </c>
       <c r="O12" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_ERD_0.01v.png</v>
       </c>
-      <c r="P12" s="6"/>
-      <c r="R12" s="15"/>
-      <c r="X12" s="16"/>
+      <c r="P12" s="5"/>
+      <c r="R12" s="14"/>
+      <c r="X12" s="15"/>
     </row>
     <row r="13" ht="28.5" customHeight="1">
       <c r="B13" s="3" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="E13" s="5" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="F13" s="4" t="s">
         <v>19</v>
@@ -1471,7 +1495,9 @@
       <c r="I13" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J13" s="3"/>
+      <c r="J13" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="K13" s="7" t="s">
         <v>24</v>
       </c>
@@ -1479,29 +1505,31 @@
       <c r="M13" s="10">
         <v>46325.0</v>
       </c>
-      <c r="N13" s="17">
+      <c r="N13" s="16">
         <v>46332.0</v>
       </c>
       <c r="O13" s="6" t="str">
         <f t="shared" si="1"/>
         <v>Final_Project_테이블 정의서_0.01v.xlsx</v>
       </c>
-      <c r="P13" s="6"/>
-      <c r="R13" s="15"/>
-      <c r="X13" s="16"/>
+      <c r="P13" s="5" t="s">
+        <v>70</v>
+      </c>
+      <c r="R13" s="14"/>
+      <c r="X13" s="15"/>
     </row>
     <row r="14" ht="28.5" customHeight="1">
       <c r="B14" s="3" t="s">
-        <v>65</v>
+        <v>71</v>
       </c>
       <c r="C14" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>67</v>
+        <v>73</v>
       </c>
       <c r="E14" s="5" t="s">
-        <v>68</v>
+        <v>74</v>
       </c>
       <c r="F14" s="4" t="s">
         <v>19</v>
@@ -1523,7 +1551,7 @@
       <c r="M14" s="10">
         <v>46329.0</v>
       </c>
-      <c r="N14" s="17">
+      <c r="N14" s="16">
         <v>46332.0</v>
       </c>
       <c r="O14" s="6" t="str">
@@ -1531,21 +1559,21 @@
         <v>Final_Project_테스트 계획서_0.01v.docx</v>
       </c>
       <c r="P14" s="6"/>
-      <c r="R14" s="15"/>
-      <c r="X14" s="16"/>
+      <c r="R14" s="14"/>
+      <c r="X14" s="15"/>
     </row>
     <row r="15" ht="28.5" customHeight="1">
       <c r="B15" s="3" t="s">
-        <v>69</v>
+        <v>75</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>66</v>
+        <v>72</v>
       </c>
       <c r="D15" s="5" t="s">
-        <v>70</v>
+        <v>76</v>
       </c>
       <c r="E15" s="5" t="s">
-        <v>71</v>
+        <v>77</v>
       </c>
       <c r="F15" s="4" t="s">
         <v>19</v>
@@ -1567,7 +1595,7 @@
       <c r="M15" s="10">
         <v>46329.0</v>
       </c>
-      <c r="N15" s="17">
+      <c r="N15" s="16">
         <v>46343.0</v>
       </c>
       <c r="O15" s="6" t="str">
@@ -1575,27 +1603,27 @@
         <v>Final_Project_테스트 케이스_0.01v.xlsx</v>
       </c>
       <c r="P15" s="6"/>
-      <c r="R15" s="15"/>
-      <c r="X15" s="16"/>
+      <c r="R15" s="14"/>
+      <c r="X15" s="15"/>
     </row>
     <row r="16" ht="28.5" customHeight="1">
       <c r="B16" s="3" t="s">
-        <v>72</v>
+        <v>78</v>
       </c>
       <c r="C16" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D16" s="5" t="s">
-        <v>74</v>
+        <v>80</v>
       </c>
       <c r="E16" s="5" t="s">
-        <v>75</v>
+        <v>81</v>
       </c>
       <c r="F16" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="G16" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="H16" s="7" t="s">
         <v>33</v>
@@ -1611,7 +1639,7 @@
       <c r="M16" s="10">
         <v>46342.0</v>
       </c>
-      <c r="N16" s="17">
+      <c r="N16" s="16">
         <v>46343.0</v>
       </c>
       <c r="O16" s="6" t="str">
@@ -1619,29 +1647,29 @@
         <v>Final_Project_관리자 매뉴얼_0.01v.docx</v>
       </c>
       <c r="P16" s="6"/>
-      <c r="R16" s="18"/>
-      <c r="S16" s="19"/>
-      <c r="T16" s="19"/>
-      <c r="U16" s="19"/>
-      <c r="V16" s="19"/>
-      <c r="W16" s="19"/>
-      <c r="X16" s="20"/>
+      <c r="R16" s="17"/>
+      <c r="S16" s="18"/>
+      <c r="T16" s="18"/>
+      <c r="U16" s="18"/>
+      <c r="V16" s="18"/>
+      <c r="W16" s="18"/>
+      <c r="X16" s="19"/>
     </row>
     <row r="17" ht="28.5" customHeight="1">
       <c r="B17" s="3" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="C17" s="4" t="s">
-        <v>73</v>
+        <v>79</v>
       </c>
       <c r="D17" s="5" t="s">
-        <v>78</v>
+        <v>84</v>
       </c>
       <c r="E17" s="5" t="s">
-        <v>79</v>
+        <v>85</v>
       </c>
       <c r="F17" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="G17" s="7" t="s">
         <v>33</v>
@@ -1660,7 +1688,7 @@
       <c r="M17" s="10">
         <v>46342.0</v>
       </c>
-      <c r="N17" s="17">
+      <c r="N17" s="16">
         <v>46343.0</v>
       </c>
       <c r="O17" s="6" t="str">
@@ -1671,16 +1699,16 @@
     </row>
     <row r="18" ht="28.5" customHeight="1">
       <c r="B18" s="3" t="s">
-        <v>80</v>
+        <v>86</v>
       </c>
       <c r="C18" s="4" t="s">
         <v>30</v>
       </c>
       <c r="D18" s="5" t="s">
-        <v>81</v>
+        <v>87</v>
       </c>
       <c r="E18" s="5" t="s">
-        <v>82</v>
+        <v>88</v>
       </c>
       <c r="F18" s="4" t="s">
         <v>19</v>
@@ -1694,7 +1722,9 @@
       <c r="I18" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="J18" s="3"/>
+      <c r="J18" s="4" t="s">
+        <v>23</v>
+      </c>
       <c r="K18" s="7" t="s">
         <v>24</v>
       </c>
@@ -1702,8 +1732,8 @@
       <c r="M18" s="10">
         <v>46323.0</v>
       </c>
-      <c r="N18" s="21">
-        <v>46325.0</v>
+      <c r="N18" s="10">
+        <v>46324.0</v>
       </c>
       <c r="O18" s="6" t="str">
         <f t="shared" si="1"/>
@@ -1713,31 +1743,35 @@
     </row>
     <row r="19" ht="28.5" customHeight="1">
       <c r="B19" s="3" t="s">
-        <v>83</v>
+        <v>89</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="D19" s="5" t="s">
-        <v>84</v>
-      </c>
-      <c r="E19" s="6"/>
+        <v>90</v>
+      </c>
+      <c r="E19" s="5" t="s">
+        <v>91</v>
+      </c>
       <c r="F19" s="3"/>
       <c r="G19" s="7" t="s">
         <v>21</v>
       </c>
       <c r="H19" s="7" t="s">
-        <v>42</v>
+        <v>46</v>
       </c>
       <c r="I19" s="3"/>
-      <c r="J19" s="3"/>
+      <c r="J19" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="K19" s="8"/>
       <c r="L19" s="8"/>
       <c r="M19" s="10">
         <v>46324.0</v>
       </c>
-      <c r="N19" s="17">
-        <v>46325.0</v>
+      <c r="N19" s="10">
+        <v>46324.0</v>
       </c>
       <c r="O19" s="6" t="str">
         <f t="shared" si="1"/>
@@ -1747,16 +1781,20 @@
     </row>
     <row r="20" ht="28.5" customHeight="1">
       <c r="B20" s="3" t="s">
-        <v>85</v>
-      </c>
-      <c r="C20" s="3"/>
+        <v>92</v>
+      </c>
+      <c r="C20" s="4" t="s">
+        <v>72</v>
+      </c>
       <c r="D20" s="5" t="s">
-        <v>86</v>
-      </c>
-      <c r="E20" s="6"/>
+        <v>93</v>
+      </c>
+      <c r="E20" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="F20" s="3"/>
       <c r="G20" s="7" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H20" s="8"/>
       <c r="I20" s="3"/>
@@ -1766,7 +1804,7 @@
       <c r="M20" s="10">
         <v>46335.0</v>
       </c>
-      <c r="N20" s="17">
+      <c r="N20" s="16">
         <v>46343.0</v>
       </c>
       <c r="O20" s="6" t="str">
@@ -1777,13 +1815,17 @@
     </row>
     <row r="21" ht="28.5" customHeight="1">
       <c r="B21" s="3" t="s">
-        <v>88</v>
-      </c>
-      <c r="C21" s="3"/>
+        <v>96</v>
+      </c>
+      <c r="C21" s="4" t="s">
+        <v>38</v>
+      </c>
       <c r="D21" s="5" t="s">
-        <v>89</v>
-      </c>
-      <c r="E21" s="6"/>
+        <v>97</v>
+      </c>
+      <c r="E21" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="F21" s="3"/>
       <c r="G21" s="7" t="s">
         <v>28</v>
@@ -1792,13 +1834,15 @@
         <v>21</v>
       </c>
       <c r="I21" s="3"/>
-      <c r="J21" s="3"/>
+      <c r="J21" s="4" t="s">
+        <v>66</v>
+      </c>
       <c r="K21" s="8"/>
       <c r="L21" s="8"/>
       <c r="M21" s="10">
         <v>46328.0</v>
       </c>
-      <c r="N21" s="17">
+      <c r="N21" s="16">
         <v>46332.0</v>
       </c>
       <c r="O21" s="6" t="str">
@@ -1809,28 +1853,30 @@
     </row>
     <row r="22" ht="28.5" customHeight="1">
       <c r="B22" s="3" t="s">
-        <v>90</v>
+        <v>99</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>91</v>
+        <v>100</v>
       </c>
       <c r="D22" s="5" t="s">
-        <v>92</v>
+        <v>101</v>
       </c>
       <c r="E22" s="5" t="s">
-        <v>93</v>
+        <v>102</v>
       </c>
       <c r="F22" s="4" t="s">
-        <v>76</v>
+        <v>82</v>
       </c>
       <c r="G22" s="7" t="s">
-        <v>87</v>
+        <v>95</v>
       </c>
       <c r="H22" s="8"/>
       <c r="I22" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="J22" s="3"/>
+      <c r="J22" s="4" t="s">
+        <v>35</v>
+      </c>
       <c r="K22" s="8"/>
       <c r="L22" s="8"/>
       <c r="M22" s="10">
@@ -1847,11 +1893,11 @@
     </row>
     <row r="23" ht="28.5" customHeight="1">
       <c r="B23" s="3" t="s">
-        <v>94</v>
+        <v>103</v>
       </c>
       <c r="C23" s="3"/>
       <c r="D23" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E23" s="6"/>
       <c r="F23" s="3"/>
@@ -1871,11 +1917,11 @@
     </row>
     <row r="24" ht="28.5" customHeight="1">
       <c r="B24" s="3" t="s">
-        <v>96</v>
+        <v>105</v>
       </c>
       <c r="C24" s="3"/>
       <c r="D24" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E24" s="6"/>
       <c r="F24" s="3"/>
@@ -1895,11 +1941,11 @@
     </row>
     <row r="25" ht="28.5" customHeight="1">
       <c r="B25" s="3" t="s">
-        <v>97</v>
+        <v>106</v>
       </c>
       <c r="C25" s="3"/>
       <c r="D25" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E25" s="6"/>
       <c r="F25" s="3"/>
@@ -1919,11 +1965,11 @@
     </row>
     <row r="26" ht="28.5" customHeight="1">
       <c r="B26" s="3" t="s">
-        <v>98</v>
+        <v>107</v>
       </c>
       <c r="C26" s="3"/>
       <c r="D26" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E26" s="6"/>
       <c r="F26" s="3"/>
@@ -1943,11 +1989,11 @@
     </row>
     <row r="27" ht="28.5" customHeight="1">
       <c r="B27" s="3" t="s">
-        <v>99</v>
+        <v>108</v>
       </c>
       <c r="C27" s="3"/>
       <c r="D27" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E27" s="6"/>
       <c r="F27" s="3"/>
@@ -1967,11 +2013,11 @@
     </row>
     <row r="28" ht="28.5" customHeight="1">
       <c r="B28" s="3" t="s">
-        <v>100</v>
+        <v>109</v>
       </c>
       <c r="C28" s="3"/>
       <c r="D28" s="5" t="s">
-        <v>95</v>
+        <v>104</v>
       </c>
       <c r="E28" s="6"/>
       <c r="F28" s="3"/>
@@ -1991,7 +2037,7 @@
     </row>
     <row r="29" ht="28.5" customHeight="1">
       <c r="B29" s="3" t="s">
-        <v>101</v>
+        <v>110</v>
       </c>
       <c r="C29" s="3"/>
       <c r="D29" s="6"/>
@@ -2013,7 +2059,7 @@
     </row>
     <row r="30" ht="28.5" customHeight="1">
       <c r="B30" s="3" t="s">
-        <v>102</v>
+        <v>111</v>
       </c>
       <c r="C30" s="3"/>
       <c r="D30" s="6"/>
@@ -2035,7 +2081,7 @@
     </row>
     <row r="31" ht="28.5" customHeight="1">
       <c r="B31" s="3" t="s">
-        <v>103</v>
+        <v>112</v>
       </c>
       <c r="C31" s="3"/>
       <c r="D31" s="6"/>
@@ -2057,7 +2103,7 @@
     </row>
     <row r="32" ht="28.5" customHeight="1">
       <c r="B32" s="3" t="s">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="C32" s="3"/>
       <c r="D32" s="6"/>
@@ -2079,7 +2125,7 @@
     </row>
     <row r="33" ht="28.5" customHeight="1">
       <c r="B33" s="3" t="s">
-        <v>105</v>
+        <v>114</v>
       </c>
       <c r="C33" s="3"/>
       <c r="D33" s="6"/>
@@ -2101,7 +2147,7 @@
     </row>
     <row r="34" ht="28.5" customHeight="1">
       <c r="B34" s="3" t="s">
-        <v>106</v>
+        <v>115</v>
       </c>
       <c r="C34" s="3"/>
       <c r="D34" s="6"/>
@@ -2123,7 +2169,7 @@
     </row>
     <row r="35" ht="28.5" customHeight="1">
       <c r="B35" s="3" t="s">
-        <v>107</v>
+        <v>116</v>
       </c>
       <c r="C35" s="3"/>
       <c r="D35" s="6"/>
@@ -2145,7 +2191,7 @@
     </row>
     <row r="36" ht="28.5" customHeight="1">
       <c r="B36" s="3" t="s">
-        <v>108</v>
+        <v>117</v>
       </c>
       <c r="C36" s="3"/>
       <c r="D36" s="6"/>
@@ -2167,7 +2213,7 @@
     </row>
     <row r="37" ht="28.5" customHeight="1">
       <c r="B37" s="3" t="s">
-        <v>109</v>
+        <v>118</v>
       </c>
       <c r="C37" s="3"/>
       <c r="D37" s="6"/>
@@ -2189,7 +2235,7 @@
     </row>
     <row r="38" ht="28.5" customHeight="1">
       <c r="B38" s="3" t="s">
-        <v>110</v>
+        <v>119</v>
       </c>
       <c r="C38" s="3"/>
       <c r="D38" s="6"/>
@@ -2211,7 +2257,7 @@
     </row>
     <row r="39" ht="28.5" customHeight="1">
       <c r="B39" s="3" t="s">
-        <v>111</v>
+        <v>120</v>
       </c>
       <c r="C39" s="3"/>
       <c r="D39" s="6"/>
@@ -2233,7 +2279,7 @@
     </row>
     <row r="40" ht="28.5" customHeight="1">
       <c r="B40" s="3" t="s">
-        <v>112</v>
+        <v>121</v>
       </c>
       <c r="C40" s="3"/>
       <c r="D40" s="6"/>
@@ -2255,7 +2301,7 @@
     </row>
     <row r="41" ht="28.5" customHeight="1">
       <c r="B41" s="3" t="s">
-        <v>113</v>
+        <v>122</v>
       </c>
       <c r="C41" s="3"/>
       <c r="D41" s="6"/>
@@ -2277,7 +2323,7 @@
     </row>
     <row r="42" ht="28.5" customHeight="1">
       <c r="B42" s="3" t="s">
-        <v>114</v>
+        <v>123</v>
       </c>
       <c r="C42" s="3"/>
       <c r="D42" s="6"/>
@@ -2299,7 +2345,7 @@
     </row>
     <row r="43" ht="28.5" customHeight="1">
       <c r="B43" s="3" t="s">
-        <v>115</v>
+        <v>124</v>
       </c>
       <c r="C43" s="3"/>
       <c r="D43" s="6"/>
@@ -2321,7 +2367,7 @@
     </row>
     <row r="44" ht="28.5" customHeight="1">
       <c r="B44" s="3" t="s">
-        <v>116</v>
+        <v>125</v>
       </c>
       <c r="C44" s="3"/>
       <c r="D44" s="6"/>
@@ -2343,7 +2389,7 @@
     </row>
     <row r="45" ht="28.5" customHeight="1">
       <c r="B45" s="3" t="s">
-        <v>117</v>
+        <v>126</v>
       </c>
       <c r="C45" s="3"/>
       <c r="D45" s="6"/>
@@ -2365,7 +2411,7 @@
     </row>
     <row r="46" ht="28.5" customHeight="1">
       <c r="B46" s="3" t="s">
-        <v>118</v>
+        <v>127</v>
       </c>
       <c r="C46" s="3"/>
       <c r="D46" s="6"/>
@@ -2387,7 +2433,7 @@
     </row>
     <row r="47" ht="28.5" customHeight="1">
       <c r="B47" s="3" t="s">
-        <v>119</v>
+        <v>128</v>
       </c>
       <c r="C47" s="3"/>
       <c r="D47" s="6"/>
@@ -2409,7 +2455,7 @@
     </row>
     <row r="48" ht="28.5" customHeight="1">
       <c r="B48" s="3" t="s">
-        <v>120</v>
+        <v>129</v>
       </c>
       <c r="C48" s="3"/>
       <c r="D48" s="6"/>
@@ -2431,7 +2477,7 @@
     </row>
     <row r="49" ht="28.5" customHeight="1">
       <c r="B49" s="3" t="s">
-        <v>121</v>
+        <v>130</v>
       </c>
       <c r="C49" s="3"/>
       <c r="D49" s="6"/>
@@ -2453,7 +2499,7 @@
     </row>
     <row r="50" ht="28.5" customHeight="1">
       <c r="B50" s="3" t="s">
-        <v>122</v>
+        <v>131</v>
       </c>
       <c r="C50" s="3"/>
       <c r="D50" s="6"/>
@@ -2475,7 +2521,7 @@
     </row>
     <row r="51" ht="28.5" customHeight="1">
       <c r="B51" s="3" t="s">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="C51" s="3"/>
       <c r="D51" s="6"/>
@@ -2497,7 +2543,7 @@
     </row>
     <row r="52" ht="28.5" customHeight="1">
       <c r="B52" s="3" t="s">
-        <v>124</v>
+        <v>133</v>
       </c>
       <c r="C52" s="3"/>
       <c r="D52" s="6"/>
@@ -2519,7 +2565,7 @@
     </row>
     <row r="53" ht="28.5" customHeight="1">
       <c r="B53" s="3" t="s">
-        <v>125</v>
+        <v>134</v>
       </c>
       <c r="C53" s="3"/>
       <c r="D53" s="6"/>
@@ -2541,7 +2587,7 @@
     </row>
     <row r="54" ht="28.5" customHeight="1">
       <c r="B54" s="3" t="s">
-        <v>126</v>
+        <v>135</v>
       </c>
       <c r="C54" s="3"/>
       <c r="D54" s="6"/>
@@ -2563,7 +2609,7 @@
     </row>
     <row r="55" ht="28.5" customHeight="1">
       <c r="B55" s="3" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="C55" s="3"/>
       <c r="D55" s="6"/>
@@ -2585,7 +2631,7 @@
     </row>
     <row r="56" ht="28.5" customHeight="1">
       <c r="B56" s="3" t="s">
-        <v>128</v>
+        <v>137</v>
       </c>
       <c r="C56" s="3"/>
       <c r="D56" s="6"/>
@@ -2607,7 +2653,7 @@
     </row>
     <row r="57" ht="28.5" customHeight="1">
       <c r="B57" s="3" t="s">
-        <v>129</v>
+        <v>138</v>
       </c>
       <c r="C57" s="3"/>
       <c r="D57" s="6"/>
@@ -2629,7 +2675,7 @@
     </row>
     <row r="58" ht="28.5" customHeight="1">
       <c r="B58" s="3" t="s">
-        <v>130</v>
+        <v>139</v>
       </c>
       <c r="C58" s="3"/>
       <c r="D58" s="6"/>
@@ -2651,7 +2697,7 @@
     </row>
     <row r="59" ht="28.5" customHeight="1">
       <c r="B59" s="3" t="s">
-        <v>131</v>
+        <v>140</v>
       </c>
       <c r="C59" s="3"/>
       <c r="D59" s="6"/>
@@ -2673,7 +2719,7 @@
     </row>
     <row r="60" ht="28.5" customHeight="1">
       <c r="B60" s="3" t="s">
-        <v>132</v>
+        <v>141</v>
       </c>
       <c r="C60" s="3"/>
       <c r="D60" s="6"/>

</xml_diff>